<commit_message>
Add demo world, logging and full test suite
apps/demo with 5 courses, 19 demo people incl. 4 product admins and learning history (seed_demo). Request IDs, global error handling, rotating local logs, secrets kept out of hosted logs. Test strategy, authorization matrix, boundary tests, OpenAPI contract check, load test, workbook with 101 manual and 220 automated tests. AI service design for review. Decisions D32-D35.
</commit_message>
<xml_diff>
--- a/docs/testing/TUTOR-test-suite.xlsx
+++ b/docs/testing/TUTOR-test-suite.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Bug log" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Automated tests'!$A$1:$G$172</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Automated tests'!$A$1:$G$186</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">'Bug log'!$A$1:$L$2</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Demo accounts'!$A$1:$F$20</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Manual cases'!$A$1:$R$96</definedName>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2663" uniqueCount="1447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2747" uniqueCount="1493">
   <si>
     <t xml:space="preserve">TUTOR test suite</t>
   </si>
@@ -2975,10 +2975,148 @@
     <t xml:space="preserve">python manage.py test apps.content.tests.RoleAdminTests.test_staff_cannot_give_themselves_admin_access --settings=config.settings.test</t>
   </si>
   <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.RequestIdTests.test_generated_and_returned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">core</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RequestIdTests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generated and returned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.RequestIdTests.test_generated_and_returned --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.RequestIdTests.test_well_formed_incoming_id_is_kept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Well formed incoming id is kept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.RequestIdTests.test_well_formed_incoming_id_is_kept --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.RequestIdTests.test_malformed_incoming_id_is_replaced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malformed incoming id is replaced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.RequestIdTests.test_malformed_incoming_id_is_replaced --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.ApiErrorShapeTests.test_error_body_carries_the_request_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ApiErrorShapeTests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error body carries the request id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.ApiErrorShapeTests.test_error_body_carries_the_request_id --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.ApiErrorShapeTests.test_unexpected_exception_is_a_clean_500_and_logged_once_with_traceback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unexpected exception is a clean 500 and logged once with traceback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.ApiErrorShapeTests.test_unexpected_exception_is_a_clean_500_and_logged_once_with_traceback --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.ApiErrorShapeTests.test_request_id_filter_stamps_records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request id filter stamps records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.ApiErrorShapeTests.test_request_id_filter_stamps_records --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.ApiErrorShapeTests.test_http404_raised_in_code_uses_the_api_shape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Http404 raised in code uses the api shape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.ApiErrorShapeTests.test_http404_raised_in_code_uses_the_api_shape --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.ApiErrorShapeTests.test_unknown_api_url_is_json_404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown api url is json 404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.ApiErrorShapeTests.test_unknown_api_url_is_json_404 --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.ApiErrorShapeTests.test_django_level_handlers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Django level handlers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.ApiErrorShapeTests.test_django_level_handlers --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.RotatingLogTests.test_console_only_without_a_log_dir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RotatingLogTests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Console only without a log dir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.RotatingLogTests.test_console_only_without_a_log_dir --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.RotatingLogTests.test_rotating_files_when_a_log_dir_is_set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rotating files when a log dir is set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.RotatingLogTests.test_rotating_files_when_a_log_dir_is_set --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.MessagingSecretsTests.test_mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MessagingSecretsTests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.MessagingSecretsTests.test_mask --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.MessagingSecretsTests.test_hosted_mode_never_logs_or_keeps_the_text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosted mode never logs or keeps the text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.MessagingSecretsTests.test_hosted_mode_never_logs_or_keeps_the_text --settings=config.settings.test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps.core.test_errors_and_logging.MessagingSecretsTests.test_outbox_is_bounded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outbox is bounded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">python manage.py test apps.core.test_errors_and_logging.MessagingSecretsTests.test_outbox_is_bounded --settings=config.settings.test</t>
+  </si>
+  <si>
     <t xml:space="preserve">apps.core.tests.DevOutboxTests.test_newest_first_and_filtered_by_recipient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">core</t>
   </si>
   <si>
     <t xml:space="preserve">DevOutboxTests</t>
@@ -5152,8 +5290,8 @@
         <v>22</v>
       </c>
       <c r="B15" s="5" t="n">
-        <f aca="false">COUNTA('Automated tests'!$A$2:$A$172)</f>
-        <v>171</v>
+        <f aca="false">COUNTA('Automated tests'!$A$2:$A$186)</f>
+        <v>185</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>23</v>
@@ -9388,7 +9526,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G172"/>
+  <dimension ref="A1:G186"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -12101,7 +12239,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="10" t="s">
         <v>967</v>
       </c>
@@ -12124,28 +12262,26 @@
     </row>
     <row r="125" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="10" t="s">
-        <v>527</v>
+        <v>970</v>
       </c>
       <c r="B125" s="10" t="s">
         <v>963</v>
       </c>
       <c r="C125" s="10" t="s">
-        <v>640</v>
+        <v>679</v>
       </c>
       <c r="D125" s="10" t="s">
-        <v>970</v>
+        <v>964</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>971</v>
       </c>
-      <c r="F125" s="10" t="s">
-        <v>522</v>
-      </c>
+      <c r="F125" s="10"/>
       <c r="G125" s="10" t="s">
         <v>972</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="10" t="s">
         <v>973</v>
       </c>
@@ -12153,7 +12289,7 @@
         <v>963</v>
       </c>
       <c r="C126" s="10" t="s">
-        <v>679</v>
+        <v>640</v>
       </c>
       <c r="D126" s="10" t="s">
         <v>974</v>
@@ -12161,14 +12297,12 @@
       <c r="E126" s="10" t="s">
         <v>975</v>
       </c>
-      <c r="F126" s="10" t="s">
-        <v>310</v>
-      </c>
+      <c r="F126" s="10"/>
       <c r="G126" s="10" t="s">
         <v>976</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="10" t="s">
         <v>977</v>
       </c>
@@ -12176,7 +12310,7 @@
         <v>963</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>679</v>
+        <v>640</v>
       </c>
       <c r="D127" s="10" t="s">
         <v>974</v>
@@ -12189,144 +12323,144 @@
         <v>979</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="10" t="s">
         <v>980</v>
       </c>
       <c r="B128" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="C128" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D128" s="10" t="s">
+        <v>974</v>
+      </c>
+      <c r="E128" s="10" t="s">
         <v>981</v>
-      </c>
-      <c r="C128" s="10" t="s">
-        <v>679</v>
-      </c>
-      <c r="D128" s="10" t="s">
-        <v>982</v>
-      </c>
-      <c r="E128" s="10" t="s">
-        <v>983</v>
       </c>
       <c r="F128" s="10"/>
       <c r="G128" s="10" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="10" t="s">
+        <v>983</v>
+      </c>
+      <c r="B129" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="C129" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D129" s="10" t="s">
+        <v>974</v>
+      </c>
+      <c r="E129" s="10" t="s">
         <v>984</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="10" t="s">
-        <v>985</v>
-      </c>
-      <c r="B129" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="C129" s="10" t="s">
-        <v>679</v>
-      </c>
-      <c r="D129" s="10" t="s">
-        <v>982</v>
-      </c>
-      <c r="E129" s="10" t="s">
-        <v>986</v>
       </c>
       <c r="F129" s="10"/>
       <c r="G129" s="10" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="10" t="s">
+        <v>986</v>
+      </c>
+      <c r="B130" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="C130" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D130" s="10" t="s">
+        <v>974</v>
+      </c>
+      <c r="E130" s="10" t="s">
         <v>987</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="10" t="s">
-        <v>988</v>
-      </c>
-      <c r="B130" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="C130" s="10" t="s">
-        <v>679</v>
-      </c>
-      <c r="D130" s="10" t="s">
-        <v>982</v>
-      </c>
-      <c r="E130" s="10" t="s">
-        <v>989</v>
       </c>
       <c r="F130" s="10"/>
       <c r="G130" s="10" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="10" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>679</v>
+        <v>640</v>
       </c>
       <c r="D131" s="10" t="s">
-        <v>982</v>
+        <v>974</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="F131" s="10"/>
       <c r="G131" s="10" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="10" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C132" s="10" t="s">
         <v>679</v>
       </c>
       <c r="D132" s="10" t="s">
-        <v>982</v>
+        <v>993</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="F132" s="10"/>
       <c r="G132" s="10" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="10" t="s">
         <v>996</v>
       </c>
-    </row>
-    <row r="133" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="10" t="s">
-        <v>997</v>
-      </c>
       <c r="B133" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C133" s="10" t="s">
         <v>679</v>
       </c>
       <c r="D133" s="10" t="s">
-        <v>982</v>
+        <v>993</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="F133" s="10"/>
       <c r="G133" s="10" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="10" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C134" s="10" t="s">
         <v>679</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>982</v>
+        <v>1000</v>
       </c>
       <c r="E134" s="10" t="s">
         <v>1001</v>
@@ -12336,18 +12470,18 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="10" t="s">
         <v>1003</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C135" s="10" t="s">
         <v>679</v>
       </c>
       <c r="D135" s="10" t="s">
-        <v>982</v>
+        <v>1000</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>1004</v>
@@ -12362,13 +12496,13 @@
         <v>1006</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C136" s="10" t="s">
         <v>679</v>
       </c>
       <c r="D136" s="10" t="s">
-        <v>982</v>
+        <v>1000</v>
       </c>
       <c r="E136" s="10" t="s">
         <v>1007</v>
@@ -12383,7 +12517,7 @@
         <v>1009</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C137" s="10" t="s">
         <v>679</v>
@@ -12394,9 +12528,7 @@
       <c r="E137" s="10" t="s">
         <v>1011</v>
       </c>
-      <c r="F137" s="10" t="s">
-        <v>480</v>
-      </c>
+      <c r="F137" s="10"/>
       <c r="G137" s="10" t="s">
         <v>1012</v>
       </c>
@@ -12406,784 +12538,1084 @@
         <v>1013</v>
       </c>
       <c r="B138" s="10" t="s">
-        <v>981</v>
+        <v>963</v>
       </c>
       <c r="C138" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="D138" s="10" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E138" s="10" t="s">
         <v>1014</v>
-      </c>
-      <c r="D138" s="10" t="s">
-        <v>1015</v>
-      </c>
-      <c r="E138" s="10" t="s">
-        <v>1016</v>
       </c>
       <c r="F138" s="10"/>
       <c r="G138" s="10" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="B139" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="C139" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D139" s="10" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E139" s="10" t="s">
         <v>1017</v>
       </c>
-    </row>
-    <row r="139" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="10" t="s">
+      <c r="F139" s="10" t="s">
+        <v>522</v>
+      </c>
+      <c r="G139" s="10" t="s">
         <v>1018</v>
       </c>
-      <c r="B139" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="C139" s="10" t="s">
-        <v>1014</v>
-      </c>
-      <c r="D139" s="10" t="s">
-        <v>1015</v>
-      </c>
-      <c r="E139" s="10" t="s">
+    </row>
+    <row r="140" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="10" t="s">
         <v>1019</v>
       </c>
-      <c r="F139" s="10"/>
-      <c r="G139" s="10" t="s">
+      <c r="B140" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="C140" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="D140" s="10" t="s">
         <v>1020</v>
       </c>
-    </row>
-    <row r="140" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="10" t="s">
+      <c r="E140" s="10" t="s">
         <v>1021</v>
       </c>
-      <c r="B140" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="C140" s="10" t="s">
-        <v>1014</v>
-      </c>
-      <c r="D140" s="10" t="s">
-        <v>1015</v>
-      </c>
-      <c r="E140" s="10" t="s">
+      <c r="F140" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="G140" s="10" t="s">
         <v>1022</v>
-      </c>
-      <c r="F140" s="10"/>
-      <c r="G140" s="10" t="s">
-        <v>1023</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="10" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B141" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="C141" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="D141" s="10" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E141" s="10" t="s">
         <v>1024</v>
-      </c>
-      <c r="B141" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="C141" s="10" t="s">
-        <v>1014</v>
-      </c>
-      <c r="D141" s="10" t="s">
-        <v>1025</v>
-      </c>
-      <c r="E141" s="10" t="s">
-        <v>253</v>
       </c>
       <c r="F141" s="10"/>
       <c r="G141" s="10" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="10" t="s">
         <v>1026</v>
       </c>
-    </row>
-    <row r="142" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="10" t="s">
-        <v>360</v>
-      </c>
       <c r="B142" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D142" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E142" s="10" t="s">
+        <v>1029</v>
+      </c>
+      <c r="F142" s="10"/>
+      <c r="G142" s="10" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="10" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B143" s="10" t="s">
         <v>1027</v>
       </c>
-      <c r="F142" s="10" t="s">
-        <v>356</v>
-      </c>
-      <c r="G142" s="10" t="s">
+      <c r="C143" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="D143" s="10" t="s">
         <v>1028</v>
       </c>
-    </row>
-    <row r="143" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="10" t="s">
-        <v>332</v>
-      </c>
-      <c r="B143" s="10" t="s">
-        <v>981</v>
-      </c>
-      <c r="C143" s="10" t="s">
-        <v>1014</v>
-      </c>
-      <c r="D143" s="10" t="s">
-        <v>1025</v>
-      </c>
       <c r="E143" s="10" t="s">
-        <v>1029</v>
-      </c>
-      <c r="F143" s="10" t="s">
-        <v>326</v>
-      </c>
+        <v>1032</v>
+      </c>
+      <c r="F143" s="10"/>
       <c r="G143" s="10" t="s">
-        <v>1030</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="10" t="s">
-        <v>1031</v>
+        <v>1034</v>
       </c>
       <c r="B144" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D144" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E144" s="10" t="s">
-        <v>645</v>
-      </c>
-      <c r="F144" s="10" t="s">
-        <v>333</v>
-      </c>
+        <v>1035</v>
+      </c>
+      <c r="F144" s="10"/>
       <c r="G144" s="10" t="s">
-        <v>1032</v>
-      </c>
-    </row>
-    <row r="145" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="10" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C145" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D145" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E145" s="10" t="s">
-        <v>1034</v>
-      </c>
-      <c r="F145" s="10" t="s">
-        <v>377</v>
-      </c>
+        <v>1038</v>
+      </c>
+      <c r="F145" s="10"/>
       <c r="G145" s="10" t="s">
-        <v>1035</v>
-      </c>
-    </row>
-    <row r="146" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="10" t="s">
-        <v>372</v>
+        <v>1040</v>
       </c>
       <c r="B146" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C146" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D146" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E146" s="10" t="s">
-        <v>1036</v>
-      </c>
-      <c r="F146" s="10" t="s">
-        <v>1037</v>
-      </c>
+        <v>1041</v>
+      </c>
+      <c r="F146" s="10"/>
       <c r="G146" s="10" t="s">
-        <v>1038</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="10" t="s">
-        <v>366</v>
+        <v>1043</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C147" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D147" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E147" s="10" t="s">
-        <v>1039</v>
-      </c>
-      <c r="F147" s="10" t="s">
-        <v>1040</v>
-      </c>
+        <v>1044</v>
+      </c>
+      <c r="F147" s="10"/>
       <c r="G147" s="10" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="10" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="B148" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C148" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D148" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E148" s="10" t="s">
-        <v>1043</v>
-      </c>
-      <c r="F148" s="10" t="s">
-        <v>1044</v>
-      </c>
+        <v>1047</v>
+      </c>
+      <c r="F148" s="10"/>
       <c r="G148" s="10" t="s">
-        <v>1045</v>
-      </c>
-    </row>
-    <row r="149" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="10" t="s">
-        <v>1046</v>
+        <v>1049</v>
       </c>
       <c r="B149" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C149" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D149" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E149" s="10" t="s">
-        <v>1047</v>
-      </c>
-      <c r="F149" s="10" t="s">
-        <v>333</v>
-      </c>
+        <v>1050</v>
+      </c>
+      <c r="F149" s="10"/>
       <c r="G149" s="10" t="s">
-        <v>1048</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="10" t="s">
-        <v>1049</v>
+        <v>1052</v>
       </c>
       <c r="B150" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C150" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D150" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="E150" s="10" t="s">
-        <v>1050</v>
-      </c>
-      <c r="F150" s="10" t="s">
-        <v>344</v>
-      </c>
+        <v>1053</v>
+      </c>
+      <c r="F150" s="10"/>
       <c r="G150" s="10" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="151" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="10" t="s">
-        <v>1052</v>
+        <v>1055</v>
       </c>
       <c r="B151" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C151" s="10" t="s">
-        <v>1014</v>
+        <v>679</v>
       </c>
       <c r="D151" s="10" t="s">
-        <v>1025</v>
+        <v>1056</v>
       </c>
       <c r="E151" s="10" t="s">
-        <v>1053</v>
-      </c>
-      <c r="F151" s="10"/>
+        <v>1057</v>
+      </c>
+      <c r="F151" s="10" t="s">
+        <v>480</v>
+      </c>
       <c r="G151" s="10" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="10" t="s">
-        <v>1055</v>
+        <v>1059</v>
       </c>
       <c r="B152" s="10" t="s">
-        <v>981</v>
+        <v>1027</v>
       </c>
       <c r="C152" s="10" t="s">
-        <v>1014</v>
+        <v>1060</v>
       </c>
       <c r="D152" s="10" t="s">
-        <v>1025</v>
+        <v>1061</v>
       </c>
       <c r="E152" s="10" t="s">
-        <v>1056</v>
-      </c>
-      <c r="F152" s="10" t="s">
-        <v>350</v>
-      </c>
+        <v>1062</v>
+      </c>
+      <c r="F152" s="10"/>
       <c r="G152" s="10" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="10" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
       <c r="B153" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C153" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D153" s="10" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="E153" s="10" t="s">
-        <v>1061</v>
+        <v>1065</v>
       </c>
       <c r="F153" s="10"/>
       <c r="G153" s="10" t="s">
-        <v>1062</v>
-      </c>
-    </row>
-    <row r="154" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="10" t="s">
-        <v>425</v>
+        <v>1067</v>
       </c>
       <c r="B154" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C154" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D154" s="10" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E154" s="10" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F154" s="10"/>
+      <c r="G154" s="10" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="10" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B155" s="10" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C155" s="10" t="s">
         <v>1060</v>
       </c>
-      <c r="E154" s="10" t="s">
-        <v>1063</v>
-      </c>
-      <c r="F154" s="10" t="s">
-        <v>421</v>
-      </c>
-      <c r="G154" s="10" t="s">
-        <v>1064</v>
-      </c>
-    </row>
-    <row r="155" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="10" t="s">
-        <v>1065</v>
-      </c>
-      <c r="B155" s="10" t="s">
-        <v>1059</v>
-      </c>
-      <c r="C155" s="10" t="s">
-        <v>818</v>
-      </c>
       <c r="D155" s="10" t="s">
-        <v>1060</v>
+        <v>1071</v>
       </c>
       <c r="E155" s="10" t="s">
-        <v>1066</v>
+        <v>253</v>
       </c>
       <c r="F155" s="10"/>
       <c r="G155" s="10" t="s">
-        <v>1067</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="10" t="s">
-        <v>1068</v>
+        <v>360</v>
       </c>
       <c r="B156" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C156" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D156" s="10" t="s">
+        <v>1071</v>
+      </c>
+      <c r="E156" s="10" t="s">
+        <v>1073</v>
+      </c>
+      <c r="F156" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="G156" s="10" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="B157" s="10" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C157" s="10" t="s">
         <v>1060</v>
       </c>
-      <c r="E156" s="10" t="s">
-        <v>1069</v>
-      </c>
-      <c r="F156" s="10"/>
-      <c r="G156" s="10" t="s">
-        <v>1070</v>
-      </c>
-    </row>
-    <row r="157" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="10" t="s">
+      <c r="D157" s="10" t="s">
         <v>1071</v>
       </c>
-      <c r="B157" s="10" t="s">
-        <v>1059</v>
-      </c>
-      <c r="C157" s="10" t="s">
-        <v>818</v>
-      </c>
-      <c r="D157" s="10" t="s">
-        <v>1060</v>
-      </c>
       <c r="E157" s="10" t="s">
-        <v>475</v>
-      </c>
-      <c r="F157" s="10"/>
+        <v>1075</v>
+      </c>
+      <c r="F157" s="10" t="s">
+        <v>326</v>
+      </c>
       <c r="G157" s="10" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="10" t="s">
-        <v>1073</v>
+        <v>1077</v>
       </c>
       <c r="B158" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C158" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D158" s="10" t="s">
-        <v>1060</v>
+        <v>1071</v>
       </c>
       <c r="E158" s="10" t="s">
-        <v>1074</v>
-      </c>
-      <c r="F158" s="10"/>
+        <v>645</v>
+      </c>
+      <c r="F158" s="10" t="s">
+        <v>333</v>
+      </c>
       <c r="G158" s="10" t="s">
-        <v>1075</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="10" t="s">
-        <v>1076</v>
+        <v>1079</v>
       </c>
       <c r="B159" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C159" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D159" s="10" t="s">
-        <v>1060</v>
+        <v>1071</v>
       </c>
       <c r="E159" s="10" t="s">
-        <v>1077</v>
-      </c>
-      <c r="F159" s="10"/>
+        <v>1080</v>
+      </c>
+      <c r="F159" s="10" t="s">
+        <v>377</v>
+      </c>
       <c r="G159" s="10" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="10" t="s">
-        <v>1079</v>
+        <v>372</v>
       </c>
       <c r="B160" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C160" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D160" s="10" t="s">
-        <v>1080</v>
+        <v>1071</v>
       </c>
       <c r="E160" s="10" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="F160" s="10" t="s">
-        <v>480</v>
+        <v>1083</v>
       </c>
       <c r="G160" s="10" t="s">
-        <v>1082</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="10" t="s">
-        <v>1083</v>
+        <v>366</v>
       </c>
       <c r="B161" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C161" s="10" t="s">
-        <v>818</v>
+        <v>1060</v>
       </c>
       <c r="D161" s="10" t="s">
-        <v>1080</v>
+        <v>1071</v>
       </c>
       <c r="E161" s="10" t="s">
-        <v>1084</v>
-      </c>
-      <c r="F161" s="10"/>
+        <v>1085</v>
+      </c>
+      <c r="F161" s="10" t="s">
+        <v>1086</v>
+      </c>
       <c r="G161" s="10" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="10" t="s">
-        <v>1086</v>
+        <v>1088</v>
       </c>
       <c r="B162" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C162" s="10" t="s">
-        <v>640</v>
+        <v>1060</v>
       </c>
       <c r="D162" s="10" t="s">
-        <v>1087</v>
+        <v>1071</v>
       </c>
       <c r="E162" s="10" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="F162" s="10" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="G162" s="10" t="s">
-        <v>1090</v>
-      </c>
-    </row>
-    <row r="163" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="10" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B163" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C163" s="10" t="s">
-        <v>640</v>
+        <v>1060</v>
       </c>
       <c r="D163" s="10" t="s">
-        <v>1087</v>
+        <v>1071</v>
       </c>
       <c r="E163" s="10" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="F163" s="10" t="s">
-        <v>387</v>
+        <v>333</v>
       </c>
       <c r="G163" s="10" t="s">
-        <v>1093</v>
-      </c>
-    </row>
-    <row r="164" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="10" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="B164" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C164" s="10" t="s">
-        <v>640</v>
+        <v>1060</v>
       </c>
       <c r="D164" s="10" t="s">
-        <v>1087</v>
+        <v>1071</v>
       </c>
       <c r="E164" s="10" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="F164" s="10" t="s">
-        <v>400</v>
+        <v>344</v>
       </c>
       <c r="G164" s="10" t="s">
-        <v>1096</v>
-      </c>
-    </row>
-    <row r="165" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="10" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B165" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C165" s="10" t="s">
-        <v>640</v>
+        <v>1060</v>
       </c>
       <c r="D165" s="10" t="s">
-        <v>1087</v>
+        <v>1071</v>
       </c>
       <c r="E165" s="10" t="s">
-        <v>1098</v>
-      </c>
-      <c r="F165" s="10" t="s">
-        <v>400</v>
-      </c>
+        <v>1099</v>
+      </c>
+      <c r="F165" s="10"/>
       <c r="G165" s="10" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="10" t="s">
-        <v>410</v>
+        <v>1101</v>
       </c>
       <c r="B166" s="10" t="s">
-        <v>1059</v>
+        <v>1027</v>
       </c>
       <c r="C166" s="10" t="s">
-        <v>640</v>
+        <v>1060</v>
       </c>
       <c r="D166" s="10" t="s">
-        <v>1087</v>
+        <v>1071</v>
       </c>
       <c r="E166" s="10" t="s">
-        <v>1100</v>
+        <v>1102</v>
       </c>
       <c r="F166" s="10" t="s">
-        <v>406</v>
+        <v>350</v>
       </c>
       <c r="G166" s="10" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="10" t="s">
-        <v>1102</v>
+        <v>1104</v>
       </c>
       <c r="B167" s="10" t="s">
-        <v>1059</v>
+        <v>1105</v>
       </c>
       <c r="C167" s="10" t="s">
-        <v>640</v>
+        <v>818</v>
       </c>
       <c r="D167" s="10" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="E167" s="10" t="s">
-        <v>1104</v>
-      </c>
-      <c r="F167" s="10" t="s">
-        <v>415</v>
-      </c>
+        <v>1107</v>
+      </c>
+      <c r="F167" s="10"/>
       <c r="G167" s="10" t="s">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="B168" s="10" t="s">
         <v>1105</v>
       </c>
-    </row>
-    <row r="168" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="B168" s="10" t="s">
-        <v>1059</v>
-      </c>
       <c r="C168" s="10" t="s">
-        <v>640</v>
+        <v>818</v>
       </c>
       <c r="D168" s="10" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="E168" s="10" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="F168" s="10" t="s">
-        <v>1107</v>
+        <v>421</v>
       </c>
       <c r="G168" s="10" t="s">
-        <v>1108</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="10" t="s">
-        <v>455</v>
+        <v>1111</v>
       </c>
       <c r="B169" s="10" t="s">
-        <v>1059</v>
+        <v>1105</v>
       </c>
       <c r="C169" s="10" t="s">
-        <v>640</v>
+        <v>818</v>
       </c>
       <c r="D169" s="10" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="E169" s="10" t="s">
-        <v>1109</v>
-      </c>
-      <c r="F169" s="10" t="s">
-        <v>451</v>
-      </c>
+        <v>1112</v>
+      </c>
+      <c r="F169" s="10"/>
       <c r="G169" s="10" t="s">
-        <v>1110</v>
-      </c>
-    </row>
-    <row r="170" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="10" t="s">
-        <v>473</v>
+        <v>1114</v>
       </c>
       <c r="B170" s="10" t="s">
-        <v>1059</v>
+        <v>1105</v>
       </c>
       <c r="C170" s="10" t="s">
-        <v>640</v>
+        <v>818</v>
       </c>
       <c r="D170" s="10" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="E170" s="10" t="s">
-        <v>1111</v>
-      </c>
-      <c r="F170" s="10" t="s">
-        <v>1112</v>
-      </c>
+        <v>1115</v>
+      </c>
+      <c r="F170" s="10"/>
       <c r="G170" s="10" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="10" t="s">
-        <v>461</v>
+        <v>1117</v>
       </c>
       <c r="B171" s="10" t="s">
-        <v>1059</v>
+        <v>1105</v>
       </c>
       <c r="C171" s="10" t="s">
-        <v>640</v>
+        <v>818</v>
       </c>
       <c r="D171" s="10" t="s">
-        <v>1114</v>
+        <v>1106</v>
       </c>
       <c r="E171" s="10" t="s">
-        <v>1115</v>
-      </c>
-      <c r="F171" s="10" t="s">
-        <v>456</v>
-      </c>
+        <v>475</v>
+      </c>
+      <c r="F171" s="10"/>
       <c r="G171" s="10" t="s">
-        <v>1116</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="10" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B172" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C172" s="10" t="s">
+        <v>818</v>
+      </c>
+      <c r="D172" s="10" t="s">
+        <v>1106</v>
+      </c>
+      <c r="E172" s="10" t="s">
+        <v>1120</v>
+      </c>
+      <c r="F172" s="10"/>
+      <c r="G172" s="10" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="10" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B173" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C173" s="10" t="s">
+        <v>818</v>
+      </c>
+      <c r="D173" s="10" t="s">
+        <v>1106</v>
+      </c>
+      <c r="E173" s="10" t="s">
+        <v>1123</v>
+      </c>
+      <c r="F173" s="10"/>
+      <c r="G173" s="10" t="s">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="10" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B174" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C174" s="10" t="s">
+        <v>818</v>
+      </c>
+      <c r="D174" s="10" t="s">
+        <v>1126</v>
+      </c>
+      <c r="E174" s="10" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F174" s="10" t="s">
+        <v>480</v>
+      </c>
+      <c r="G174" s="10" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="10" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B175" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C175" s="10" t="s">
+        <v>818</v>
+      </c>
+      <c r="D175" s="10" t="s">
+        <v>1126</v>
+      </c>
+      <c r="E175" s="10" t="s">
+        <v>1130</v>
+      </c>
+      <c r="F175" s="10"/>
+      <c r="G175" s="10" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="10" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B176" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C176" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D176" s="10" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E176" s="10" t="s">
+        <v>1134</v>
+      </c>
+      <c r="F176" s="10" t="s">
+        <v>1135</v>
+      </c>
+      <c r="G176" s="10" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="10" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B177" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C177" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D177" s="10" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E177" s="10" t="s">
+        <v>1138</v>
+      </c>
+      <c r="F177" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="G177" s="10" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="10" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B178" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C178" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D178" s="10" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E178" s="10" t="s">
+        <v>1141</v>
+      </c>
+      <c r="F178" s="10" t="s">
+        <v>400</v>
+      </c>
+      <c r="G178" s="10" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="10" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B179" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C179" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D179" s="10" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E179" s="10" t="s">
+        <v>1144</v>
+      </c>
+      <c r="F179" s="10" t="s">
+        <v>400</v>
+      </c>
+      <c r="G179" s="10" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="B180" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C180" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D180" s="10" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E180" s="10" t="s">
+        <v>1146</v>
+      </c>
+      <c r="F180" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="G180" s="10" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="10" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B181" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C181" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D181" s="10" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E181" s="10" t="s">
+        <v>1150</v>
+      </c>
+      <c r="F181" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="G181" s="10" t="s">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="B182" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C182" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D182" s="10" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E182" s="10" t="s">
+        <v>1152</v>
+      </c>
+      <c r="F182" s="10" t="s">
+        <v>1153</v>
+      </c>
+      <c r="G182" s="10" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="10" t="s">
+        <v>455</v>
+      </c>
+      <c r="B183" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C183" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D183" s="10" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E183" s="10" t="s">
+        <v>1155</v>
+      </c>
+      <c r="F183" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="G183" s="10" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="10" t="s">
+        <v>473</v>
+      </c>
+      <c r="B184" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C184" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D184" s="10" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E184" s="10" t="s">
+        <v>1157</v>
+      </c>
+      <c r="F184" s="10" t="s">
+        <v>1158</v>
+      </c>
+      <c r="G184" s="10" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="B185" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C185" s="10" t="s">
+        <v>640</v>
+      </c>
+      <c r="D185" s="10" t="s">
+        <v>1160</v>
+      </c>
+      <c r="E185" s="10" t="s">
+        <v>1161</v>
+      </c>
+      <c r="F185" s="10" t="s">
+        <v>456</v>
+      </c>
+      <c r="G185" s="10" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="10" t="s">
         <v>466</v>
       </c>
-      <c r="B172" s="10" t="s">
-        <v>1059</v>
-      </c>
-      <c r="C172" s="10" t="s">
+      <c r="B186" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C186" s="10" t="s">
         <v>640</v>
       </c>
-      <c r="D172" s="10" t="s">
-        <v>1114</v>
-      </c>
-      <c r="E172" s="10" t="s">
+      <c r="D186" s="10" t="s">
+        <v>1160</v>
+      </c>
+      <c r="E186" s="10" t="s">
         <v>463</v>
       </c>
-      <c r="F172" s="10" t="s">
+      <c r="F186" s="10" t="s">
         <v>462</v>
       </c>
-      <c r="G172" s="10" t="s">
-        <v>1117</v>
+      <c r="G186" s="10" t="s">
+        <v>1163</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G172"/>
+  <autoFilter ref="A1:G186"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -13210,604 +13642,604 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>1118</v>
+        <v>1164</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1119</v>
+        <v>1165</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>1120</v>
+        <v>1166</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>1121</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1123</v>
+        <v>1169</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>1124</v>
+        <v>1170</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1126</v>
+        <v>1172</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1127</v>
+        <v>1173</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1128</v>
+        <v>1174</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1129</v>
+        <v>1175</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1130</v>
+        <v>1176</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1131</v>
+        <v>1177</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1132</v>
+        <v>1178</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1133</v>
+        <v>1179</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1134</v>
+        <v>1180</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1135</v>
+        <v>1181</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1136</v>
+        <v>1182</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>1137</v>
+        <v>1183</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1138</v>
+        <v>1184</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>1139</v>
+        <v>1185</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>1140</v>
+        <v>1186</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>1141</v>
+        <v>1187</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>1142</v>
+        <v>1188</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>1143</v>
+        <v>1189</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>1144</v>
+        <v>1190</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>1145</v>
+        <v>1191</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>1146</v>
+        <v>1192</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>1147</v>
+        <v>1193</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>1148</v>
+        <v>1194</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>1149</v>
+        <v>1195</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>1150</v>
+        <v>1196</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>1151</v>
+        <v>1197</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>320</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>1152</v>
+        <v>1198</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1122</v>
+        <v>1168</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>1153</v>
+        <v>1199</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>1154</v>
+        <v>1200</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>1125</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>77</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>1156</v>
+        <v>1202</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>77</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>1158</v>
+        <v>1204</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1159</v>
+        <v>1205</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>1139</v>
+        <v>1185</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>1160</v>
+        <v>1206</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>1141</v>
+        <v>1187</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>1161</v>
+        <v>1207</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>1162</v>
+        <v>1208</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>1163</v>
+        <v>1209</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>1164</v>
+        <v>1210</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>1165</v>
+        <v>1211</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>1166</v>
+        <v>1212</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>1167</v>
+        <v>1213</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>1168</v>
+        <v>1214</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>1169</v>
+        <v>1215</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>1170</v>
+        <v>1216</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>147</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>1171</v>
+        <v>1217</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>1172</v>
+        <v>1218</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>1173</v>
+        <v>1219</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>1174</v>
+        <v>1220</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>1175</v>
+        <v>1221</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1176</v>
+        <v>1222</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>1177</v>
+        <v>1223</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>1178</v>
+        <v>1224</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>1179</v>
+        <v>1225</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>1180</v>
+        <v>1226</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>1181</v>
+        <v>1227</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>1182</v>
+        <v>1228</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>1183</v>
+        <v>1229</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>1184</v>
+        <v>1230</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>1185</v>
+        <v>1231</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>1186</v>
+        <v>1232</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>1187</v>
+        <v>1233</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>1188</v>
+        <v>1234</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>1189</v>
+        <v>1235</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>1190</v>
+        <v>1236</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>1191</v>
+        <v>1237</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>1192</v>
+        <v>1238</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>1193</v>
+        <v>1239</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>1194</v>
+        <v>1240</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>1195</v>
+        <v>1241</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>1196</v>
+        <v>1242</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>1197</v>
+        <v>1243</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>1198</v>
+        <v>1244</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>1199</v>
+        <v>1245</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>1200</v>
+        <v>1246</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>1201</v>
+        <v>1247</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>1155</v>
+        <v>1201</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>1202</v>
+        <v>1248</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>1147</v>
+        <v>1193</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>1157</v>
+        <v>1203</v>
       </c>
     </row>
   </sheetData>
@@ -13843,28 +14275,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>1203</v>
+        <v>1249</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>46</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>1204</v>
+        <v>1250</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>1205</v>
+        <v>1251</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>1206</v>
+        <v>1252</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>1207</v>
+        <v>1253</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>1208</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13872,16 +14304,16 @@
         <v>100</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>1210</v>
+        <v>1256</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>1212</v>
+        <v>1258</v>
       </c>
       <c r="F2" s="10" t="n">
         <v>5</v>
@@ -13899,16 +14331,16 @@
         <v>94</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1213</v>
+        <v>1259</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>1214</v>
+        <v>1260</v>
       </c>
       <c r="F3" s="10" t="n">
         <v>3</v>
@@ -13926,16 +14358,16 @@
         <v>136</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1215</v>
+        <v>1261</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>1216</v>
+        <v>1262</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>3</v>
@@ -13953,16 +14385,16 @@
         <v>143</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1217</v>
+        <v>1263</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>1218</v>
+        <v>1264</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>3</v>
@@ -13980,16 +14412,16 @@
         <v>518</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1219</v>
+        <v>1265</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>1220</v>
+        <v>1266</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>2</v>
@@ -14007,13 +14439,13 @@
         <v>186</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1221</v>
+        <v>1267</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>184</v>
@@ -14034,13 +14466,13 @@
         <v>198</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>1222</v>
+        <v>1268</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>196</v>
@@ -14058,16 +14490,16 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1223</v>
+        <v>1269</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>1224</v>
+        <v>1270</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>1225</v>
+        <v>1271</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10" t="n">
@@ -14086,13 +14518,13 @@
         <v>233</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>1209</v>
+        <v>1255</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>1226</v>
+        <v>1272</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>1227</v>
+        <v>1273</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>231</v>
@@ -14110,16 +14542,16 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>1228</v>
+        <v>1274</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>1229</v>
+        <v>1275</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>1230</v>
+        <v>1276</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10" t="n">
@@ -14138,16 +14570,16 @@
         <v>255</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>1229</v>
+        <v>1275</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>1231</v>
+        <v>1277</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>1232</v>
+        <v>1278</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>4</v>
@@ -14165,16 +14597,16 @@
         <v>292</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>1229</v>
+        <v>1275</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>1233</v>
+        <v>1279</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>1234</v>
+        <v>1280</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>2</v>
@@ -14192,13 +14624,13 @@
         <v>530</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>1235</v>
+        <v>1281</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>1236</v>
+        <v>1282</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>528</v>
@@ -14219,16 +14651,16 @@
         <v>384</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>1235</v>
+        <v>1281</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>1237</v>
+        <v>1283</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>1238</v>
+        <v>1284</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>2</v>
@@ -14246,16 +14678,16 @@
         <v>217</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>1235</v>
+        <v>1281</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>1239</v>
+        <v>1285</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>1240</v>
+        <v>1286</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>1241</v>
+        <v>1287</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>4</v>
@@ -14273,16 +14705,16 @@
         <v>335</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>1243</v>
+        <v>1289</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>1244</v>
+        <v>1290</v>
       </c>
       <c r="F17" s="10" t="n">
         <v>3</v>
@@ -14300,16 +14732,16 @@
         <v>341</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>1245</v>
+        <v>1291</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>1246</v>
+        <v>1292</v>
       </c>
       <c r="F18" s="10" t="n">
         <v>3</v>
@@ -14327,13 +14759,13 @@
         <v>417</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>1247</v>
+        <v>1293</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>415</v>
@@ -14354,16 +14786,16 @@
         <v>428</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>1248</v>
+        <v>1294</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>1249</v>
+        <v>1295</v>
       </c>
       <c r="F20" s="10" t="n">
         <v>3</v>
@@ -14378,19 +14810,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>1250</v>
+        <v>1296</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>1251</v>
+        <v>1297</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>1252</v>
+        <v>1298</v>
       </c>
       <c r="F21" s="10" t="n">
         <v>2</v>
@@ -14408,16 +14840,16 @@
         <v>469</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>1253</v>
+        <v>1299</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>1254</v>
+        <v>1300</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>2</v>
@@ -14435,13 +14867,13 @@
         <v>476</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>1255</v>
+        <v>1301</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>1211</v>
+        <v>1257</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>474</v>
@@ -14459,16 +14891,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>1256</v>
+        <v>1302</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>1242</v>
+        <v>1288</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>1257</v>
+        <v>1303</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="10" t="n">
@@ -14484,16 +14916,16 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>1259</v>
+        <v>1305</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>1260</v>
+        <v>1306</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>1261</v>
+        <v>1307</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10" t="n">
@@ -14509,16 +14941,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>1262</v>
+        <v>1308</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>1260</v>
+        <v>1306</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>1263</v>
+        <v>1309</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="10" t="n">
@@ -14534,16 +14966,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>1264</v>
+        <v>1310</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>1260</v>
+        <v>1306</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>1265</v>
+        <v>1311</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="10" t="n">
@@ -14559,16 +14991,16 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>1266</v>
+        <v>1312</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>1267</v>
+        <v>1313</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>1268</v>
+        <v>1314</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="10" t="n">
@@ -14584,16 +15016,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>1269</v>
+        <v>1315</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>1267</v>
+        <v>1313</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>1270</v>
+        <v>1316</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E29" s="10"/>
       <c r="F29" s="10" t="n">
@@ -14609,16 +15041,16 @@
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>1271</v>
+        <v>1317</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1272</v>
+        <v>1318</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>1273</v>
+        <v>1319</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>1258</v>
+        <v>1304</v>
       </c>
       <c r="E30" s="10"/>
       <c r="F30" s="10" t="n">
@@ -14637,13 +15069,13 @@
         <v>524</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>1274</v>
+        <v>1320</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>1275</v>
+        <v>1321</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>1276</v>
+        <v>1322</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>522</v>
@@ -14664,16 +15096,16 @@
         <v>317</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>1277</v>
+        <v>1323</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>1278</v>
+        <v>1324</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>1280</v>
+        <v>1326</v>
       </c>
       <c r="F32" s="10" t="n">
         <v>2</v>
@@ -14691,16 +15123,16 @@
         <v>80</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>1277</v>
+        <v>1323</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>1281</v>
+        <v>1327</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>1282</v>
+        <v>1328</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>2</v>
@@ -14718,13 +15150,13 @@
         <v>512</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>1277</v>
+        <v>1323</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>1283</v>
+        <v>1329</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E34" s="10" t="s">
         <v>510</v>
@@ -14745,16 +15177,16 @@
         <v>555</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>1277</v>
+        <v>1323</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>1284</v>
+        <v>1330</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>1285</v>
+        <v>1331</v>
       </c>
       <c r="F35" s="10" t="n">
         <v>3</v>
@@ -14772,16 +15204,16 @@
         <v>369</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>1277</v>
+        <v>1323</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>1286</v>
+        <v>1332</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>1287</v>
+        <v>1333</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>4</v>
@@ -14799,13 +15231,13 @@
         <v>550</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>1288</v>
+        <v>1334</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>1289</v>
+        <v>1335</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>548</v>
@@ -14823,16 +15255,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>1290</v>
+        <v>1336</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>1288</v>
+        <v>1334</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>1291</v>
+        <v>1337</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E38" s="10"/>
       <c r="F38" s="10" t="n">
@@ -14848,16 +15280,16 @@
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>1292</v>
+        <v>1338</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>1293</v>
+        <v>1339</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>1294</v>
+        <v>1340</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E39" s="10"/>
       <c r="F39" s="10" t="n">
@@ -14876,16 +15308,16 @@
         <v>67</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>1295</v>
+        <v>1341</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>1296</v>
+        <v>1342</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>1297</v>
+        <v>1343</v>
       </c>
       <c r="F40" s="10" t="n">
         <v>2</v>
@@ -14900,16 +15332,16 @@
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>1298</v>
+        <v>1344</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>1299</v>
+        <v>1345</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>1300</v>
+        <v>1346</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E41" s="10"/>
       <c r="F41" s="10" t="n">
@@ -14925,16 +15357,16 @@
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>1301</v>
+        <v>1347</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>1293</v>
+        <v>1339</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>1302</v>
+        <v>1348</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E42" s="10"/>
       <c r="F42" s="10" t="n">
@@ -14950,16 +15382,16 @@
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>1303</v>
+        <v>1349</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>1304</v>
+        <v>1350</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>1305</v>
+        <v>1351</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="10" t="n">
@@ -14975,16 +15407,16 @@
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
-        <v>1306</v>
+        <v>1352</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>1307</v>
+        <v>1353</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>1308</v>
+        <v>1354</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E44" s="10"/>
       <c r="F44" s="10" t="n">
@@ -15003,16 +15435,16 @@
         <v>352</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>1309</v>
+        <v>1355</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>1310</v>
+        <v>1356</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>1279</v>
+        <v>1325</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>1311</v>
+        <v>1357</v>
       </c>
       <c r="F45" s="10" t="n">
         <v>2</v>
@@ -15066,402 +15498,402 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>1312</v>
+        <v>1358</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1313</v>
+        <v>1359</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>1314</v>
+        <v>1360</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>1315</v>
+        <v>1361</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>1316</v>
+        <v>1362</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>1317</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1318</v>
+        <v>1364</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1319</v>
+        <v>1365</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>1320</v>
+        <v>1366</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>1321</v>
+        <v>1367</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>1322</v>
+        <v>1368</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>1323</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1324</v>
+        <v>1370</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1325</v>
+        <v>1371</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1326</v>
+        <v>1372</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>1327</v>
+        <v>1373</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>1328</v>
+        <v>1374</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>1329</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1330</v>
+        <v>1376</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1331</v>
+        <v>1377</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1332</v>
+        <v>1378</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>1333</v>
+        <v>1379</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>1334</v>
+        <v>1380</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>1335</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1336</v>
+        <v>1382</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1337</v>
+        <v>1383</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1338</v>
+        <v>1384</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>1339</v>
+        <v>1385</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>1340</v>
+        <v>1386</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>1341</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1342</v>
+        <v>1388</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1343</v>
+        <v>1389</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1344</v>
+        <v>1390</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>1345</v>
+        <v>1391</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>1346</v>
+        <v>1392</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>1347</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1348</v>
+        <v>1394</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1349</v>
+        <v>1395</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1350</v>
+        <v>1396</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>1351</v>
+        <v>1397</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>1352</v>
+        <v>1398</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>1353</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1354</v>
+        <v>1400</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1355</v>
+        <v>1401</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>1356</v>
+        <v>1402</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>1357</v>
+        <v>1403</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>1358</v>
+        <v>1404</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>1359</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1360</v>
+        <v>1406</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1361</v>
+        <v>1407</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>1362</v>
+        <v>1408</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>1363</v>
+        <v>1409</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>1364</v>
+        <v>1410</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>1365</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>1366</v>
+        <v>1412</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>1367</v>
+        <v>1413</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>1368</v>
+        <v>1414</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>1369</v>
+        <v>1415</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>1370</v>
+        <v>1416</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>1371</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>1372</v>
+        <v>1418</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>1373</v>
+        <v>1419</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>1374</v>
+        <v>1420</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>1375</v>
+        <v>1421</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>1376</v>
+        <v>1422</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>1377</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>1378</v>
+        <v>1424</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>1379</v>
+        <v>1425</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>1380</v>
+        <v>1426</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>1381</v>
+        <v>1427</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>1382</v>
+        <v>1428</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>1383</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>1384</v>
+        <v>1430</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>1385</v>
+        <v>1431</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>1386</v>
+        <v>1432</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>1387</v>
+        <v>1433</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>1388</v>
+        <v>1434</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>1389</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>1390</v>
+        <v>1436</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>1391</v>
+        <v>1437</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>1392</v>
+        <v>1438</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>1393</v>
+        <v>1439</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>1394</v>
+        <v>1440</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>1395</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1396</v>
+        <v>1442</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>1397</v>
+        <v>1443</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>1398</v>
+        <v>1444</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>1399</v>
+        <v>1445</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>1400</v>
+        <v>1446</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>1401</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1402</v>
+        <v>1448</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>1403</v>
+        <v>1449</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>1404</v>
+        <v>1450</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>1405</v>
+        <v>1451</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>1406</v>
+        <v>1452</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>1407</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1408</v>
+        <v>1454</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>1409</v>
+        <v>1455</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>1410</v>
+        <v>1456</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>1411</v>
+        <v>1457</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>1412</v>
+        <v>1458</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>1413</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1414</v>
+        <v>1460</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>1415</v>
+        <v>1461</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>1416</v>
+        <v>1462</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>1417</v>
+        <v>1463</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>1418</v>
+        <v>1464</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>1419</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1420</v>
+        <v>1466</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>1421</v>
+        <v>1467</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>1422</v>
+        <v>1468</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>1423</v>
+        <v>1469</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>1424</v>
+        <v>1470</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>1425</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1426</v>
+        <v>1472</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1427</v>
+        <v>1473</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>1428</v>
+        <v>1474</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>1429</v>
+        <v>1475</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>1430</v>
+        <v>1476</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>1431</v>
+        <v>1477</v>
       </c>
     </row>
   </sheetData>
@@ -15502,7 +15934,7 @@
         <v>60</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1432</v>
+        <v>1478</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>48</v>
@@ -15514,19 +15946,19 @@
         <v>51</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>1433</v>
+        <v>1479</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>1434</v>
+        <v>1480</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>1435</v>
+        <v>1481</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>1436</v>
+        <v>1482</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>1437</v>
+        <v>1483</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>57</v>
@@ -15537,40 +15969,40 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>1438</v>
+        <v>1484</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>441</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1439</v>
+        <v>1485</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>1440</v>
+        <v>1486</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>68</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>1441</v>
+        <v>1487</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>1442</v>
+        <v>1488</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>1443</v>
+        <v>1489</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>1444</v>
+        <v>1490</v>
       </c>
       <c r="J2" s="12" t="n">
         <v>46296</v>
       </c>
       <c r="K2" s="11" t="s">
-        <v>1445</v>
+        <v>1491</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>1446</v>
+        <v>1492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>